<commit_message>
Prompt coach live test: plant known answers in SUS-1 to SUS-3
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp6bbiPXfwDc65dz8hiGei
</commit_message>
<xml_diff>
--- a/prompt-coach/research/live-tests/fixtures/sus_ghg_inventory.xlsx
+++ b/prompt-coach/research/live-tests/fixtures/sus_ghg_inventory.xlsx
@@ -397,17 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Category</v>
       </c>
       <c r="B1" t="str">
-        <v>FY2024</v>
+        <v>FY2024 (tCO2e)</v>
       </c>
       <c r="C1" t="str">
-        <v>FY2025</v>
+        <v>FY2025 (tCO2e)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Note</v>
       </c>
     </row>
     <row r="2">
@@ -454,9 +457,34 @@
         <v>88</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Upstream transport</v>
+      </c>
+      <c r="B6">
+        <v>150</v>
+      </c>
+      <c r="C6">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Leased assets</v>
+      </c>
+      <c r="B7">
+        <v>60</v>
+      </c>
+      <c r="C7">
+        <v>0.061</v>
+      </c>
+      <c r="D7" t="str">
+        <v>FY2025 in ktCO2e</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>